<commit_message>
reduced rod to 36 in for free shipping
</commit_message>
<xml_diff>
--- a/SYS_DEV/Columbia/V0/V0.7/v0.7.0/BOM-SPECIES-Columbia-v0.7.0.xlsx
+++ b/SYS_DEV/Columbia/V0/V0.7/v0.7.0/BOM-SPECIES-Columbia-v0.7.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Smart-Penetrometer-with-Edge-Computing-and-Intelligent-Embedded-Systems\SYS_DEV\Columbia\V0\V0.7\v0.7.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D57FC3C6-30BF-49BA-8AE3-593B8E8FC7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26AD5620-D63B-4800-8CD2-2459157146DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-150" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -74,9 +74,6 @@
     <t>https://www.grainger.com/product/ABS-Tube-Stock-3-ft-Lg-60CY12?opr=ODOH&amp;analytics=FM:Order%20History</t>
   </si>
   <si>
-    <t>https://www.grainger.com/product/360-Brass-Rod-1-4-in-Outside-803H36?opr=ILOF</t>
-  </si>
-  <si>
     <t>ABS Tube Stock: 3 ft Lg, 1/4 in Inside Dia, 1/2 in Outside Dia, 0.13 in Wall Thick, Opaque, Black</t>
   </si>
   <si>
@@ -86,9 +83,6 @@
     <t>longest piece with free shipping on USC contract</t>
   </si>
   <si>
-    <t>360 Brass Rod: 1/4 in Outside Dia, 4 ft Overall Lg, H02, Mill, 45,000 psi Yield Strength</t>
-  </si>
-  <si>
     <t>https://www.grainger.com/product/SHRINK-KON-Heat-Shrink-Tubing-0-75-in-3KH60?opr=ILOF</t>
   </si>
   <si>
@@ -147,6 +141,12 @@
   </si>
   <si>
     <t>inner brass rod - spike probe</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/360-Brass-Rod-1-4-in-Outside-803H35?opr=ILOF</t>
+  </si>
+  <si>
+    <t>360 Brass Rod: 1/4 in Outside Dia, 36 in Overall Lg, H02, Mill, 45,000 psi Yield Strength, Inch</t>
   </si>
 </sst>
 </file>
@@ -599,10 +599,10 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>3</v>
@@ -611,7 +611,7 @@
         <v>0</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>4</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2">
@@ -651,20 +651,20 @@
         <v>6.57</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="2"/>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2">
@@ -678,18 +678,18 @@
         <v>2.0562499999999999</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2">
@@ -703,7 +703,7 @@
         <v>2.26953</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>11</v>
@@ -713,10 +713,10 @@
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2">
@@ -731,17 +731,17 @@
       </c>
       <c r="G5" s="6"/>
       <c r="H5" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="5"/>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2">
@@ -756,18 +756,18 @@
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2">
@@ -781,13 +781,13 @@
         <v>9.98E-2</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
@@ -1082,15 +1082,14 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H4" r:id="rId1" xr:uid="{A2E1C8C8-6A04-46E2-AC51-28CA639AB5C3}"/>
-    <hyperlink ref="H3" r:id="rId2" xr:uid="{DF7A5359-89D1-4378-AEAB-FD422BE4C122}"/>
-    <hyperlink ref="H5" r:id="rId3" xr:uid="{3552A92A-EFA4-4FB0-92CC-E82180001E88}"/>
-    <hyperlink ref="I6" r:id="rId4" xr:uid="{FA8CF8E9-26AB-43B4-820A-5FF0ECE212F3}"/>
-    <hyperlink ref="H6" r:id="rId5" xr:uid="{B0CFF966-AF61-4A69-82E7-3D5DCE98FD10}"/>
-    <hyperlink ref="H2" r:id="rId6" xr:uid="{4C1B4732-A388-4A05-ACD7-7F60A4FA52BC}"/>
-    <hyperlink ref="I7" r:id="rId7" display="https://www.homedepot.com/p/Gorilla-8-oz-Original-Glue-50008A/100204163" xr:uid="{3687080D-7764-4AE9-84DA-09203FC30570}"/>
-    <hyperlink ref="H7" r:id="rId8" xr:uid="{2DA22F02-0B2C-466B-8EB5-68D61876C27A}"/>
+    <hyperlink ref="H5" r:id="rId2" xr:uid="{3552A92A-EFA4-4FB0-92CC-E82180001E88}"/>
+    <hyperlink ref="I6" r:id="rId3" xr:uid="{FA8CF8E9-26AB-43B4-820A-5FF0ECE212F3}"/>
+    <hyperlink ref="H6" r:id="rId4" xr:uid="{B0CFF966-AF61-4A69-82E7-3D5DCE98FD10}"/>
+    <hyperlink ref="H2" r:id="rId5" xr:uid="{4C1B4732-A388-4A05-ACD7-7F60A4FA52BC}"/>
+    <hyperlink ref="I7" r:id="rId6" display="https://www.homedepot.com/p/Gorilla-8-oz-Original-Glue-50008A/100204163" xr:uid="{3687080D-7764-4AE9-84DA-09203FC30570}"/>
+    <hyperlink ref="H7" r:id="rId7" xr:uid="{2DA22F02-0B2C-466B-8EB5-68D61876C27A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId9"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>